<commit_message>
Added analog filtering and fixed audio noise
</commit_message>
<xml_diff>
--- a/Electronics/PCBs/Main/BOM.xlsx
+++ b/Electronics/PCBs/Main/BOM.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="BOM_Board1_PCB-V1_2026-04-29" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="BOM_Board1_PCB-V1_2026-05-11" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -124,25 +124,40 @@
     <t>5</t>
   </si>
   <si>
+    <t>220pF</t>
+  </si>
+  <si>
+    <t>CASIG,CSPKRG,CSPKRV</t>
+  </si>
+  <si>
+    <t>C0603</t>
+  </si>
+  <si>
+    <t>CL10B221KB8NNNC</t>
+  </si>
+  <si>
+    <t>SAMSUNG(三星)</t>
+  </si>
+  <si>
+    <t>C1603</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
     <t>10uF</t>
   </si>
   <si>
     <t>CAVDD2,CCH340,CDVDD2,CESP2</t>
   </si>
   <si>
-    <t>C0603</t>
-  </si>
-  <si>
     <t>CL10A106MA8NRNC</t>
   </si>
   <si>
-    <t>SAMSUNG(三星)</t>
-  </si>
-  <si>
     <t>C96446</t>
   </si>
   <si>
-    <t>6</t>
+    <t>7</t>
   </si>
   <si>
     <t>100nF</t>
@@ -160,7 +175,7 @@
     <t>C14663</t>
   </si>
   <si>
-    <t>7</t>
+    <t>8</t>
   </si>
   <si>
     <t>15pF</t>
@@ -175,7 +190,7 @@
     <t>C1644</t>
   </si>
   <si>
-    <t>8</t>
+    <t>9</t>
   </si>
   <si>
     <t>CH340C</t>
@@ -190,7 +205,7 @@
     <t>C84681</t>
   </si>
   <si>
-    <t>9</t>
+    <t>10</t>
   </si>
   <si>
     <t>1uF</t>
@@ -205,7 +220,7 @@
     <t>C1592</t>
   </si>
   <si>
-    <t>10</t>
+    <t>11</t>
   </si>
   <si>
     <t>10nF</t>
@@ -223,7 +238,7 @@
     <t>C57112</t>
   </si>
   <si>
-    <t>11</t>
+    <t>12</t>
   </si>
   <si>
     <t>B4B-PH-K-S(LF)(SN)</t>
@@ -238,7 +253,7 @@
     <t>C131334</t>
   </si>
   <si>
-    <t>12</t>
+    <t>13</t>
   </si>
   <si>
     <t>B2B-PH-K-S(LF)(SN)</t>
@@ -253,7 +268,7 @@
     <t>C131337</t>
   </si>
   <si>
-    <t>13</t>
+    <t>14</t>
   </si>
   <si>
     <t>B5B-PH-K-S(LF)(SN)</t>
@@ -268,7 +283,7 @@
     <t>C157993</t>
   </si>
   <si>
-    <t>14</t>
+    <t>15</t>
   </si>
   <si>
     <t>B7B-PH-K-S(LF)(SN)</t>
@@ -283,7 +298,7 @@
     <t>C157981</t>
   </si>
   <si>
-    <t>15</t>
+    <t>16</t>
   </si>
   <si>
     <t>470uF</t>
@@ -302,21 +317,6 @@
   </si>
   <si>
     <t>C5154</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>220pF</t>
-  </si>
-  <si>
-    <t>CSPKRG,CSPKRV</t>
-  </si>
-  <si>
-    <t>CL10B221KB8NNNC</t>
-  </si>
-  <si>
-    <t>C1603</t>
   </si>
   <si>
     <t>17</t>
@@ -1119,7 +1119,7 @@
         <v>36</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C6" t="s">
         <v>37</v>
@@ -1151,7 +1151,7 @@
         <v>43</v>
       </c>
       <c r="B7">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C7" t="s">
         <v>44</v>
@@ -1169,10 +1169,10 @@
         <v>46</v>
       </c>
       <c r="H7" t="s">
+        <v>41</v>
+      </c>
+      <c r="I7" t="s">
         <v>47</v>
-      </c>
-      <c r="I7" t="s">
-        <v>48</v>
       </c>
       <c r="J7" t="s">
         <v>17</v>
@@ -1180,28 +1180,28 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
         <v>49</v>
       </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>50</v>
-      </c>
-      <c r="D8" t="s">
-        <v>51</v>
       </c>
       <c r="E8" t="s">
         <v>39</v>
       </c>
       <c r="F8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G8" t="s">
+        <v>51</v>
+      </c>
+      <c r="H8" t="s">
         <v>52</v>
-      </c>
-      <c r="H8" t="s">
-        <v>41</v>
       </c>
       <c r="I8" t="s">
         <v>53</v>
@@ -1221,19 +1221,19 @@
         <v>55</v>
       </c>
       <c r="D9" t="s">
+        <v>56</v>
+      </c>
+      <c r="E9" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9" t="s">
         <v>55</v>
       </c>
-      <c r="E9" t="s">
-        <v>56</v>
-      </c>
-      <c r="F9" t="s">
-        <v>14</v>
-      </c>
       <c r="G9" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H9" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="I9" t="s">
         <v>58</v>
@@ -1247,25 +1247,25 @@
         <v>59</v>
       </c>
       <c r="B10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C10" t="s">
         <v>60</v>
       </c>
       <c r="D10" t="s">
+        <v>60</v>
+      </c>
+      <c r="E10" t="s">
         <v>61</v>
       </c>
-      <c r="E10" t="s">
-        <v>39</v>
-      </c>
       <c r="F10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" t="s">
         <v>60</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>62</v>
-      </c>
-      <c r="H10" t="s">
-        <v>41</v>
       </c>
       <c r="I10" t="s">
         <v>63</v>
@@ -1279,7 +1279,7 @@
         <v>64</v>
       </c>
       <c r="B11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C11" t="s">
         <v>65</v>
@@ -1297,10 +1297,10 @@
         <v>67</v>
       </c>
       <c r="H11" t="s">
+        <v>41</v>
+      </c>
+      <c r="I11" t="s">
         <v>68</v>
-      </c>
-      <c r="I11" t="s">
-        <v>69</v>
       </c>
       <c r="J11" t="s">
         <v>17</v>
@@ -1308,28 +1308,28 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>69</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
         <v>70</v>
       </c>
-      <c r="B12">
-        <v>4</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>71</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
+        <v>39</v>
+      </c>
+      <c r="F12" t="s">
+        <v>70</v>
+      </c>
+      <c r="G12" t="s">
         <v>72</v>
       </c>
-      <c r="E12" t="s">
+      <c r="H12" t="s">
         <v>73</v>
-      </c>
-      <c r="F12" t="s">
-        <v>14</v>
-      </c>
-      <c r="G12" t="s">
-        <v>71</v>
-      </c>
-      <c r="H12" t="s">
-        <v>28</v>
       </c>
       <c r="I12" t="s">
         <v>74</v>
@@ -1343,7 +1343,7 @@
         <v>75</v>
       </c>
       <c r="B13">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C13" t="s">
         <v>76</v>
@@ -1407,7 +1407,7 @@
         <v>85</v>
       </c>
       <c r="B15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" t="s">
         <v>86</v>
@@ -1451,16 +1451,16 @@
         <v>93</v>
       </c>
       <c r="F16" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" t="s">
         <v>91</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
+        <v>28</v>
+      </c>
+      <c r="I16" t="s">
         <v>94</v>
-      </c>
-      <c r="H16" t="s">
-        <v>95</v>
-      </c>
-      <c r="I16" t="s">
-        <v>96</v>
       </c>
       <c r="J16" t="s">
         <v>17</v>
@@ -1468,28 +1468,28 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>95</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
+        <v>96</v>
+      </c>
+      <c r="D17" t="s">
         <v>97</v>
       </c>
-      <c r="B17">
-        <v>2</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="E17" t="s">
         <v>98</v>
       </c>
-      <c r="D17" t="s">
+      <c r="F17" t="s">
+        <v>96</v>
+      </c>
+      <c r="G17" t="s">
         <v>99</v>
       </c>
-      <c r="E17" t="s">
-        <v>39</v>
-      </c>
-      <c r="F17" t="s">
-        <v>98</v>
-      </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>100</v>
-      </c>
-      <c r="H17" t="s">
-        <v>41</v>
       </c>
       <c r="I17" t="s">
         <v>101</v>
@@ -1681,7 +1681,7 @@
         <v>136</v>
       </c>
       <c r="H23" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="I23" t="s">
         <v>137</v>

</xml_diff>

<commit_message>
Moved SG90 pins to motor driver & added main board fuse
</commit_message>
<xml_diff>
--- a/Electronics/PCBs/Main/BOM.xlsx
+++ b/Electronics/PCBs/Main/BOM.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="BOM_Board1_PCB-V1_2026-05-11" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="BOM_Board1_PCB_2026-05-27" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="197">
   <si>
     <t>No.</t>
   </si>
@@ -256,10 +256,25 @@
     <t>13</t>
   </si>
   <si>
+    <t>B5B-PH-K-S(LF)(SN)</t>
+  </si>
+  <si>
+    <t>CN-MOTORS,MIC</t>
+  </si>
+  <si>
+    <t>CONN-TH_B5B-PH-K-S-LF-SN</t>
+  </si>
+  <si>
+    <t>C157993</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
     <t>B2B-PH-K-S(LF)(SN)</t>
   </si>
   <si>
-    <t>CN-EARS,CN-POWER</t>
+    <t>CN-POWER</t>
   </si>
   <si>
     <t>CONN-TH_B2B-PH-K-S</t>
@@ -268,21 +283,6 @@
     <t>C131337</t>
   </si>
   <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>B5B-PH-K-S(LF)(SN)</t>
-  </si>
-  <si>
-    <t>CN-MOTORS,MIC</t>
-  </si>
-  <si>
-    <t>CONN-TH_B5B-PH-K-S-LF-SN</t>
-  </si>
-  <si>
-    <t>C157993</t>
-  </si>
-  <si>
     <t>15</t>
   </si>
   <si>
@@ -340,6 +340,21 @@
     <t>18</t>
   </si>
   <si>
+    <t>SMAJ5.0A</t>
+  </si>
+  <si>
+    <t>D3</t>
+  </si>
+  <si>
+    <t>RUILON(瑞隆源)</t>
+  </si>
+  <si>
+    <t>C10758</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
     <t>ESP32-S3-WROOM-1U-N16R8</t>
   </si>
   <si>
@@ -355,7 +370,22 @@
     <t>C3013946</t>
   </si>
   <si>
-    <t>19</t>
+    <t>20</t>
+  </si>
+  <si>
+    <t>SMD1812P150TF/16</t>
+  </si>
+  <si>
+    <t>F1</t>
+  </si>
+  <si>
+    <t>F1812</t>
+  </si>
+  <si>
+    <t>C20810</t>
+  </si>
+  <si>
+    <t>21</t>
   </si>
   <si>
     <t>BLM18SG121TN1D</t>
@@ -373,7 +403,7 @@
     <t>C113030</t>
   </si>
   <si>
-    <t>20</t>
+    <t>22</t>
   </si>
   <si>
     <t>PAM8406DR</t>
@@ -391,7 +421,7 @@
     <t>C86270</t>
   </si>
   <si>
-    <t>21</t>
+    <t>23</t>
   </si>
   <si>
     <t>S8050 J3Y(RANGE:200-350)</t>
@@ -409,7 +439,7 @@
     <t>C2146</t>
   </si>
   <si>
-    <t>22</t>
+    <t>24</t>
   </si>
   <si>
     <t>1kΩ</t>
@@ -427,7 +457,7 @@
     <t>C22548</t>
   </si>
   <si>
-    <t>23</t>
+    <t>25</t>
   </si>
   <si>
     <t>10kΩ</t>
@@ -445,7 +475,7 @@
     <t>C25804</t>
   </si>
   <si>
-    <t>24</t>
+    <t>26</t>
   </si>
   <si>
     <t>22kΩ</t>
@@ -460,7 +490,7 @@
     <t>C31850</t>
   </si>
   <si>
-    <t>25</t>
+    <t>27</t>
   </si>
   <si>
     <t>4.7kΩ</t>
@@ -475,7 +505,7 @@
     <t>C23162</t>
   </si>
   <si>
-    <t>26</t>
+    <t>28</t>
   </si>
   <si>
     <t>2.2kΩ</t>
@@ -490,7 +520,7 @@
     <t>C4190</t>
   </si>
   <si>
-    <t>27</t>
+    <t>29</t>
   </si>
   <si>
     <t>1.25mm-2P ZZ-MS</t>
@@ -508,7 +538,7 @@
     <t>C5368706</t>
   </si>
   <si>
-    <t>28</t>
+    <t>30</t>
   </si>
   <si>
     <t>TYPE-C16PIN</t>
@@ -523,7 +553,7 @@
     <t>C393939</t>
   </si>
   <si>
-    <t>29</t>
+    <t>31</t>
   </si>
   <si>
     <t>USBLC6-2SC6</t>
@@ -541,7 +571,7 @@
     <t>C7519</t>
   </si>
   <si>
-    <t>30</t>
+    <t>32</t>
   </si>
   <si>
     <t>XC6206-1.2V</t>
@@ -559,7 +589,7 @@
     <t>C49446790</t>
   </si>
   <si>
-    <t>31</t>
+    <t>33</t>
   </si>
   <si>
     <t>XC6206-2.8V</t>
@@ -948,7 +978,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="10" width="20" customWidth="1"/>
@@ -1407,7 +1437,7 @@
         <v>85</v>
       </c>
       <c r="B15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C15" t="s">
         <v>86</v>
@@ -1544,7 +1574,7 @@
         <v>110</v>
       </c>
       <c r="E19" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="F19" t="s">
         <v>14</v>
@@ -1553,10 +1583,10 @@
         <v>109</v>
       </c>
       <c r="H19" t="s">
+        <v>111</v>
+      </c>
+      <c r="I19" t="s">
         <v>112</v>
-      </c>
-      <c r="I19" t="s">
-        <v>113</v>
       </c>
       <c r="J19" t="s">
         <v>17</v>
@@ -1564,31 +1594,31 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>113</v>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20" t="s">
         <v>114</v>
       </c>
-      <c r="B20">
-        <v>3</v>
-      </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>115</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>116</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" t="s">
+        <v>114</v>
+      </c>
+      <c r="H20" t="s">
         <v>117</v>
       </c>
-      <c r="F20" t="s">
-        <v>14</v>
-      </c>
-      <c r="G20" t="s">
-        <v>115</v>
-      </c>
-      <c r="H20" t="s">
+      <c r="I20" t="s">
         <v>118</v>
-      </c>
-      <c r="I20" t="s">
-        <v>119</v>
       </c>
       <c r="J20" t="s">
         <v>17</v>
@@ -1596,31 +1626,31 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B21">
         <v>1</v>
       </c>
       <c r="C21" t="s">
+        <v>120</v>
+      </c>
+      <c r="D21" t="s">
         <v>121</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>122</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21" t="s">
+        <v>120</v>
+      </c>
+      <c r="H21" t="s">
+        <v>111</v>
+      </c>
+      <c r="I21" t="s">
         <v>123</v>
-      </c>
-      <c r="F21" t="s">
-        <v>14</v>
-      </c>
-      <c r="G21" t="s">
-        <v>121</v>
-      </c>
-      <c r="H21" t="s">
-        <v>124</v>
-      </c>
-      <c r="I21" t="s">
-        <v>125</v>
       </c>
       <c r="J21" t="s">
         <v>17</v>
@@ -1628,31 +1658,31 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22">
+        <v>3</v>
+      </c>
+      <c r="C22" t="s">
+        <v>125</v>
+      </c>
+      <c r="D22" t="s">
         <v>126</v>
       </c>
-      <c r="B22">
-        <v>2</v>
-      </c>
-      <c r="C22" t="s">
+      <c r="E22" t="s">
         <v>127</v>
       </c>
-      <c r="D22" t="s">
+      <c r="F22" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" t="s">
+        <v>125</v>
+      </c>
+      <c r="H22" t="s">
         <v>128</v>
       </c>
-      <c r="E22" t="s">
+      <c r="I22" t="s">
         <v>129</v>
-      </c>
-      <c r="F22" t="s">
-        <v>14</v>
-      </c>
-      <c r="G22" t="s">
-        <v>127</v>
-      </c>
-      <c r="H22" t="s">
-        <v>130</v>
-      </c>
-      <c r="I22" t="s">
-        <v>131</v>
       </c>
       <c r="J22" t="s">
         <v>17</v>
@@ -1660,31 +1690,31 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>130</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>131</v>
+      </c>
+      <c r="D23" t="s">
         <v>132</v>
       </c>
-      <c r="B23">
-        <v>2</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="E23" t="s">
         <v>133</v>
       </c>
-      <c r="D23" t="s">
+      <c r="F23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G23" t="s">
+        <v>131</v>
+      </c>
+      <c r="H23" t="s">
         <v>134</v>
       </c>
-      <c r="E23" t="s">
+      <c r="I23" t="s">
         <v>135</v>
-      </c>
-      <c r="F23" t="s">
-        <v>133</v>
-      </c>
-      <c r="G23" t="s">
-        <v>136</v>
-      </c>
-      <c r="H23" t="s">
-        <v>52</v>
-      </c>
-      <c r="I23" t="s">
-        <v>137</v>
       </c>
       <c r="J23" t="s">
         <v>17</v>
@@ -1692,31 +1722,31 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>136</v>
+      </c>
+      <c r="B24">
+        <v>2</v>
+      </c>
+      <c r="C24" t="s">
+        <v>137</v>
+      </c>
+      <c r="D24" t="s">
         <v>138</v>
       </c>
-      <c r="B24">
-        <v>3</v>
-      </c>
-      <c r="C24" t="s">
+      <c r="E24" t="s">
         <v>139</v>
       </c>
-      <c r="D24" t="s">
+      <c r="F24" t="s">
+        <v>14</v>
+      </c>
+      <c r="G24" t="s">
+        <v>137</v>
+      </c>
+      <c r="H24" t="s">
         <v>140</v>
       </c>
-      <c r="E24" t="s">
-        <v>135</v>
-      </c>
-      <c r="F24" t="s">
-        <v>139</v>
-      </c>
-      <c r="G24" t="s">
+      <c r="I24" t="s">
         <v>141</v>
-      </c>
-      <c r="H24" t="s">
-        <v>142</v>
-      </c>
-      <c r="I24" t="s">
-        <v>143</v>
       </c>
       <c r="J24" t="s">
         <v>17</v>
@@ -1724,31 +1754,31 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>142</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>143</v>
+      </c>
+      <c r="D25" t="s">
         <v>144</v>
       </c>
-      <c r="B25">
-        <v>1</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="E25" t="s">
         <v>145</v>
       </c>
-      <c r="D25" t="s">
+      <c r="F25" t="s">
+        <v>143</v>
+      </c>
+      <c r="G25" t="s">
         <v>146</v>
       </c>
-      <c r="E25" t="s">
-        <v>135</v>
-      </c>
-      <c r="F25" t="s">
-        <v>145</v>
-      </c>
-      <c r="G25" t="s">
+      <c r="H25" t="s">
+        <v>52</v>
+      </c>
+      <c r="I25" t="s">
         <v>147</v>
-      </c>
-      <c r="H25" t="s">
-        <v>142</v>
-      </c>
-      <c r="I25" t="s">
-        <v>148</v>
       </c>
       <c r="J25" t="s">
         <v>17</v>
@@ -1756,28 +1786,28 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>148</v>
+      </c>
+      <c r="B26">
+        <v>3</v>
+      </c>
+      <c r="C26" t="s">
         <v>149</v>
       </c>
-      <c r="B26">
-        <v>1</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>150</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
+        <v>145</v>
+      </c>
+      <c r="F26" t="s">
+        <v>149</v>
+      </c>
+      <c r="G26" t="s">
         <v>151</v>
       </c>
-      <c r="E26" t="s">
-        <v>135</v>
-      </c>
-      <c r="F26" t="s">
-        <v>150</v>
-      </c>
-      <c r="G26" t="s">
+      <c r="H26" t="s">
         <v>152</v>
-      </c>
-      <c r="H26" t="s">
-        <v>142</v>
       </c>
       <c r="I26" t="s">
         <v>153</v>
@@ -1791,7 +1821,7 @@
         <v>154</v>
       </c>
       <c r="B27">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C27" t="s">
         <v>155</v>
@@ -1800,7 +1830,7 @@
         <v>156</v>
       </c>
       <c r="E27" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="F27" t="s">
         <v>155</v>
@@ -1809,7 +1839,7 @@
         <v>157</v>
       </c>
       <c r="H27" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="I27" t="s">
         <v>158</v>
@@ -1832,19 +1862,19 @@
         <v>161</v>
       </c>
       <c r="E28" t="s">
+        <v>145</v>
+      </c>
+      <c r="F28" t="s">
+        <v>160</v>
+      </c>
+      <c r="G28" t="s">
         <v>162</v>
       </c>
-      <c r="F28" t="s">
-        <v>14</v>
-      </c>
-      <c r="G28" t="s">
-        <v>160</v>
-      </c>
       <c r="H28" t="s">
+        <v>152</v>
+      </c>
+      <c r="I28" t="s">
         <v>163</v>
-      </c>
-      <c r="I28" t="s">
-        <v>164</v>
       </c>
       <c r="J28" t="s">
         <v>17</v>
@@ -1852,31 +1882,31 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>164</v>
+      </c>
+      <c r="B29">
+        <v>4</v>
+      </c>
+      <c r="C29" t="s">
         <v>165</v>
       </c>
-      <c r="B29">
-        <v>1</v>
-      </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
         <v>166</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
+        <v>145</v>
+      </c>
+      <c r="F29" t="s">
+        <v>165</v>
+      </c>
+      <c r="G29" t="s">
         <v>167</v>
       </c>
-      <c r="E29" t="s">
+      <c r="H29" t="s">
+        <v>152</v>
+      </c>
+      <c r="I29" t="s">
         <v>168</v>
-      </c>
-      <c r="F29" t="s">
-        <v>14</v>
-      </c>
-      <c r="G29" t="s">
-        <v>166</v>
-      </c>
-      <c r="H29" t="s">
-        <v>163</v>
-      </c>
-      <c r="I29" t="s">
-        <v>169</v>
       </c>
       <c r="J29" t="s">
         <v>17</v>
@@ -1884,31 +1914,31 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B30">
         <v>1</v>
       </c>
       <c r="C30" t="s">
+        <v>170</v>
+      </c>
+      <c r="D30" t="s">
         <v>171</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>172</v>
       </c>
-      <c r="E30" t="s">
+      <c r="F30" t="s">
+        <v>14</v>
+      </c>
+      <c r="G30" t="s">
+        <v>170</v>
+      </c>
+      <c r="H30" t="s">
         <v>173</v>
       </c>
-      <c r="F30" t="s">
-        <v>14</v>
-      </c>
-      <c r="G30" t="s">
-        <v>171</v>
-      </c>
-      <c r="H30" t="s">
+      <c r="I30" t="s">
         <v>174</v>
-      </c>
-      <c r="I30" t="s">
-        <v>175</v>
       </c>
       <c r="J30" t="s">
         <v>17</v>
@@ -1916,31 +1946,31 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B31">
         <v>1</v>
       </c>
       <c r="C31" t="s">
+        <v>176</v>
+      </c>
+      <c r="D31" t="s">
         <v>177</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>178</v>
       </c>
-      <c r="E31" t="s">
+      <c r="F31" t="s">
+        <v>14</v>
+      </c>
+      <c r="G31" t="s">
+        <v>176</v>
+      </c>
+      <c r="H31" t="s">
+        <v>173</v>
+      </c>
+      <c r="I31" t="s">
         <v>179</v>
-      </c>
-      <c r="F31" t="s">
-        <v>14</v>
-      </c>
-      <c r="G31" t="s">
-        <v>177</v>
-      </c>
-      <c r="H31" t="s">
-        <v>180</v>
-      </c>
-      <c r="I31" t="s">
-        <v>181</v>
       </c>
       <c r="J31" t="s">
         <v>17</v>
@@ -1948,38 +1978,102 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B32">
         <v>1</v>
       </c>
       <c r="C32" t="s">
+        <v>181</v>
+      </c>
+      <c r="D32" t="s">
+        <v>182</v>
+      </c>
+      <c r="E32" t="s">
         <v>183</v>
       </c>
-      <c r="D32" t="s">
+      <c r="F32" t="s">
+        <v>14</v>
+      </c>
+      <c r="G32" t="s">
+        <v>181</v>
+      </c>
+      <c r="H32" t="s">
         <v>184</v>
       </c>
-      <c r="E32" t="s">
+      <c r="I32" t="s">
         <v>185</v>
       </c>
-      <c r="F32" t="s">
-        <v>14</v>
-      </c>
-      <c r="G32" t="s">
-        <v>183</v>
-      </c>
-      <c r="H32" t="s">
-        <v>180</v>
-      </c>
-      <c r="I32" t="s">
+      <c r="J32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>186</v>
       </c>
-      <c r="J32" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+      <c r="B33">
+        <v>1</v>
+      </c>
+      <c r="C33" t="s">
+        <v>187</v>
+      </c>
+      <c r="D33" t="s">
+        <v>188</v>
+      </c>
+      <c r="E33" t="s">
+        <v>189</v>
+      </c>
+      <c r="F33" t="s">
+        <v>14</v>
+      </c>
+      <c r="G33" t="s">
+        <v>187</v>
+      </c>
+      <c r="H33" t="s">
+        <v>190</v>
+      </c>
+      <c r="I33" t="s">
+        <v>191</v>
+      </c>
+      <c r="J33" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>192</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>193</v>
+      </c>
+      <c r="D34" t="s">
+        <v>194</v>
+      </c>
+      <c r="E34" t="s">
+        <v>195</v>
+      </c>
+      <c r="F34" t="s">
+        <v>14</v>
+      </c>
+      <c r="G34" t="s">
+        <v>193</v>
+      </c>
+      <c r="H34" t="s">
+        <v>190</v>
+      </c>
+      <c r="I34" t="s">
+        <v>196</v>
+      </c>
+      <c r="J34" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>